<commit_message>
Add comprehensive tests for assertion message improvements, Excel export functionality, and signal bit width parsing
- Implemented `test_enter_key_fix.py` to verify the fix for Enter key navigation in the wizard.
- Created `test_excel_export.py` to test Excel export functionality with signal bit width parsing.
- Developed `test_final_messages.py` to display improved assertion messages with clarity and order.
- Added `test_parameter_fix.py` to ensure correct parameter resolution and extraction from module data.
- Introduced `test_pulse_width_display.py` to verify the display of PulseWidth assertions.
- Implemented `test_signal_bit_width.py` to test signal width parsing and formatting.
- Created `test_signal_integration.py` to simulate the complete flow of signal bit width parsing and Excel export.
- Added edge case tests in `test_signal_integration.py` to validate signal name extraction and bit width formatting.
</commit_message>
<xml_diff>
--- a/out/sessions/sync_signal-20251109_004011/sync_signal.xlsx
+++ b/out/sessions/sync_signal-20251109_004011/sync_signal.xlsx
@@ -2550,7 +2550,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N11"/>
+  <dimension ref="B1:N11"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="16.5"/>
   <cols>
     <col width="9" customWidth="1" style="53" min="1" max="1"/>
@@ -5798,7 +5798,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:S136"/>
+  <dimension ref="B3:S136"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="4.375" customWidth="1" min="1" max="1"/>
@@ -5811,8 +5811,6 @@
     <col width="18.625" customWidth="1" style="44" min="19" max="19"/>
   </cols>
   <sheetData>
-    <row r="1"/>
-    <row r="2"/>
     <row r="3" ht="19.5" customHeight="1">
       <c r="G3" t="inlineStr">
         <is>
@@ -6362,62 +6360,6 @@
       <c r="R31" s="83" t="n"/>
       <c r="S31" s="82" t="n"/>
     </row>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
-    <row r="80"/>
-    <row r="81"/>
-    <row r="82"/>
-    <row r="83"/>
-    <row r="84"/>
-    <row r="85"/>
-    <row r="86"/>
-    <row r="87"/>
     <row r="88">
       <c r="H88" s="43" t="n"/>
       <c r="J88" s="44" t="n"/>
@@ -6642,7 +6584,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:AP118"/>
+  <dimension ref="B2:AP118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="4.375" customWidth="1" min="1" max="1"/>
@@ -6679,7 +6621,6 @@
       </c>
       <c r="E3" s="258" t="n"/>
     </row>
-    <row r="4"/>
     <row r="5" ht="21" customHeight="1">
       <c r="B5" s="72" t="n"/>
       <c r="C5" s="165" t="inlineStr">
@@ -7810,7 +7751,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:AF53"/>
+  <dimension ref="B2:AF53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="4.375" customWidth="1" min="1" max="1"/>
@@ -8387,7 +8328,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:O39"/>
+  <dimension ref="B2:O39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="4.375" customWidth="1" min="1" max="1"/>
@@ -8757,7 +8698,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="C1:T55"/>
+  <dimension ref="C2:T55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="4.375" customWidth="1" min="1" max="1"/>
@@ -9243,7 +9184,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:V36"/>
+  <dimension ref="B3:V36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="4.375" customWidth="1" min="1" max="1"/>
@@ -9270,8 +9211,6 @@
     <col width="3.125" customWidth="1" min="23" max="23"/>
   </cols>
   <sheetData>
-    <row r="1"/>
-    <row r="2"/>
     <row r="3" ht="19.5" customHeight="1">
       <c r="B3" s="123" t="inlineStr">
         <is>

</xml_diff>